<commit_message>
Add Simulation tab (no import duty / single battery set), rack ex-tarifario scenario, deal structure v3 deck
- New Simulation/Simulacao tab in both summary workbooks (added by
  add_simulation_sheet.py, existing tabs untouched): two switches (remove
  II from everything; 1 vs 2 battery sets) plus a fixed four-scenario
  comparison, all live formulas linked to the P&L tab. Shows that removing
  ALL import duty cuts the Final Client Price by ~US$149k while the local
  output taxes (PIS/COFINS + ICMS + IPI) add ~US$461k (about 3.1x more);
  no II + 1 battery set still lands ~34% above the US$900k reference.
- Rack ex-tarifario scenario workbooks (EN/PT): LXA+MCA+GoLinc+PTC+
  connectors as one PN with II zeroed, optional Fastbrake, editable groups.
- Deal structure deck v3 (EN/PT): Pathfinder Iron Ore Car wording, Supermetal
  TP as an open question, 12 open tax questions; generated by
  build_deal_structure_deck.py.
- ppt-builder agent added under .claude/agents/.
</commit_message>
<xml_diff>
--- a/Pathfinder_Cost_Summary_EN.xlsx
+++ b/Pathfinder_Cost_Summary_EN.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item List" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary (P&amp;L)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Calc Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Item List'!$A$3:$M$165</definedName>
@@ -20,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="\R\$\ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -110,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,6 +139,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9514,4 +9526,1122 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIMULATION - what really makes the Pathfinder Iron Ore Car expensive</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Change the two yellow switches; the comparison table on the right never depends on them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>SWITCHES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Remove import duty (II) from everything?  (1 = yes, 0 = no)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Battery sets  (2 = current BOM, 1 = a single set)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>BASE VALUES (read from the P&amp;L tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Exchange rate</t>
+        </is>
+      </c>
+      <c r="B9" s="22">
+        <f>'Executive Summary (P&amp;L)'!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Deal Margin (TDM)</t>
+        </is>
+      </c>
+      <c r="B10" s="17">
+        <f>'Executive Summary (P&amp;L)'!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PIS/COFINS</t>
+        </is>
+      </c>
+      <c r="B11" s="17">
+        <f>'Executive Summary (P&amp;L)'!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ICMS</t>
+        </is>
+      </c>
+      <c r="B12" s="17">
+        <f>'Executive Summary (P&amp;L)'!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IPI</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>'Executive Summary (P&amp;L)'!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>US domestic reference price (USD, input)</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>SCENARIOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Selected (switches) - BRL</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Selected (switches) - USD</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Base (current) - BRL</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Base (current) - USD</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>No import duty (II) - BRL</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>No import duty (II) - USD</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>1 battery set - BRL</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>1 battery set - USD</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>No II + 1 battery set - BRL</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>No II + 1 battery set - USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Raw cost - imported items</t>
+        </is>
+      </c>
+      <c r="B19" s="24">
+        <f>$B$48+$C$48*($B$6)</f>
+        <v/>
+      </c>
+      <c r="C19" s="25">
+        <f>B19/$B$9</f>
+        <v/>
+      </c>
+      <c r="D19" s="4">
+        <f>$B$48+$C$48*(2)</f>
+        <v/>
+      </c>
+      <c r="E19" s="3">
+        <f>D19/$B$9</f>
+        <v/>
+      </c>
+      <c r="F19" s="4">
+        <f>$B$48+$C$48*(2)</f>
+        <v/>
+      </c>
+      <c r="G19" s="3">
+        <f>F19/$B$9</f>
+        <v/>
+      </c>
+      <c r="H19" s="4">
+        <f>$B$48+$C$48*(1)</f>
+        <v/>
+      </c>
+      <c r="I19" s="3">
+        <f>H19/$B$9</f>
+        <v/>
+      </c>
+      <c r="J19" s="4">
+        <f>$B$48+$C$48*(1)</f>
+        <v/>
+      </c>
+      <c r="K19" s="3">
+        <f>J19/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Raw cost - PAC items</t>
+        </is>
+      </c>
+      <c r="B20" s="24">
+        <f>$B$49</f>
+        <v/>
+      </c>
+      <c r="C20" s="25">
+        <f>B20/$B$9</f>
+        <v/>
+      </c>
+      <c r="D20" s="4">
+        <f>$B$49</f>
+        <v/>
+      </c>
+      <c r="E20" s="3">
+        <f>D20/$B$9</f>
+        <v/>
+      </c>
+      <c r="F20" s="4">
+        <f>$B$49</f>
+        <v/>
+      </c>
+      <c r="G20" s="3">
+        <f>F20/$B$9</f>
+        <v/>
+      </c>
+      <c r="H20" s="4">
+        <f>$B$49</f>
+        <v/>
+      </c>
+      <c r="I20" s="3">
+        <f>H20/$B$9</f>
+        <v/>
+      </c>
+      <c r="J20" s="4">
+        <f>$B$49</f>
+        <v/>
+      </c>
+      <c r="K20" s="3">
+        <f>J20/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TP - Transfer Price</t>
+        </is>
+      </c>
+      <c r="B21" s="24">
+        <f>$B$50+$C$50*($B$6)</f>
+        <v/>
+      </c>
+      <c r="C21" s="25">
+        <f>B21/$B$9</f>
+        <v/>
+      </c>
+      <c r="D21" s="4">
+        <f>$B$50+$C$50*(2)</f>
+        <v/>
+      </c>
+      <c r="E21" s="3">
+        <f>D21/$B$9</f>
+        <v/>
+      </c>
+      <c r="F21" s="4">
+        <f>$B$50+$C$50*(2)</f>
+        <v/>
+      </c>
+      <c r="G21" s="3">
+        <f>F21/$B$9</f>
+        <v/>
+      </c>
+      <c r="H21" s="4">
+        <f>$B$50+$C$50*(1)</f>
+        <v/>
+      </c>
+      <c r="I21" s="3">
+        <f>H21/$B$9</f>
+        <v/>
+      </c>
+      <c r="J21" s="4">
+        <f>$B$50+$C$50*(1)</f>
+        <v/>
+      </c>
+      <c r="K21" s="3">
+        <f>J21/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>International freight</t>
+        </is>
+      </c>
+      <c r="B22" s="24">
+        <f>$B$51+$C$51*($B$6)</f>
+        <v/>
+      </c>
+      <c r="C22" s="25">
+        <f>B22/$B$9</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>$B$51+$C$51*(2)</f>
+        <v/>
+      </c>
+      <c r="E22" s="3">
+        <f>D22/$B$9</f>
+        <v/>
+      </c>
+      <c r="F22" s="4">
+        <f>$B$51+$C$51*(2)</f>
+        <v/>
+      </c>
+      <c r="G22" s="3">
+        <f>F22/$B$9</f>
+        <v/>
+      </c>
+      <c r="H22" s="4">
+        <f>$B$51+$C$51*(1)</f>
+        <v/>
+      </c>
+      <c r="I22" s="3">
+        <f>H22/$B$9</f>
+        <v/>
+      </c>
+      <c r="J22" s="4">
+        <f>$B$51+$C$51*(1)</f>
+        <v/>
+      </c>
+      <c r="K22" s="3">
+        <f>J22/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>II - Import duty</t>
+        </is>
+      </c>
+      <c r="B23" s="24">
+        <f>($B$52+$C$52*($B$6))*(1-($B$5))</f>
+        <v/>
+      </c>
+      <c r="C23" s="25">
+        <f>B23/$B$9</f>
+        <v/>
+      </c>
+      <c r="D23" s="4">
+        <f>($B$52+$C$52*(2))*(1-(0))</f>
+        <v/>
+      </c>
+      <c r="E23" s="3">
+        <f>D23/$B$9</f>
+        <v/>
+      </c>
+      <c r="F23" s="4">
+        <f>($B$52+$C$52*(2))*(1-(1))</f>
+        <v/>
+      </c>
+      <c r="G23" s="3">
+        <f>F23/$B$9</f>
+        <v/>
+      </c>
+      <c r="H23" s="4">
+        <f>($B$52+$C$52*(1))*(1-(0))</f>
+        <v/>
+      </c>
+      <c r="I23" s="3">
+        <f>H23/$B$9</f>
+        <v/>
+      </c>
+      <c r="J23" s="4">
+        <f>($B$52+$C$52*(1))*(1-(1))</f>
+        <v/>
+      </c>
+      <c r="K23" s="3">
+        <f>J23/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Domestic freight</t>
+        </is>
+      </c>
+      <c r="B24" s="24">
+        <f>$B$53</f>
+        <v/>
+      </c>
+      <c r="C24" s="25">
+        <f>B24/$B$9</f>
+        <v/>
+      </c>
+      <c r="D24" s="4">
+        <f>$B$53</f>
+        <v/>
+      </c>
+      <c r="E24" s="3">
+        <f>D24/$B$9</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>$B$53</f>
+        <v/>
+      </c>
+      <c r="G24" s="3">
+        <f>F24/$B$9</f>
+        <v/>
+      </c>
+      <c r="H24" s="4">
+        <f>$B$53</f>
+        <v/>
+      </c>
+      <c r="I24" s="3">
+        <f>H24/$B$9</f>
+        <v/>
+      </c>
+      <c r="J24" s="4">
+        <f>$B$53</f>
+        <v/>
+      </c>
+      <c r="K24" s="3">
+        <f>J24/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Supermetal - refurbishment / integration</t>
+        </is>
+      </c>
+      <c r="B25" s="24">
+        <f>$B$54</f>
+        <v/>
+      </c>
+      <c r="C25" s="25">
+        <f>B25/$B$9</f>
+        <v/>
+      </c>
+      <c r="D25" s="4">
+        <f>$B$54</f>
+        <v/>
+      </c>
+      <c r="E25" s="3">
+        <f>D25/$B$9</f>
+        <v/>
+      </c>
+      <c r="F25" s="4">
+        <f>$B$54</f>
+        <v/>
+      </c>
+      <c r="G25" s="3">
+        <f>F25/$B$9</f>
+        <v/>
+      </c>
+      <c r="H25" s="4">
+        <f>$B$54</f>
+        <v/>
+      </c>
+      <c r="I25" s="3">
+        <f>H25/$B$9</f>
+        <v/>
+      </c>
+      <c r="J25" s="4">
+        <f>$B$54</f>
+        <v/>
+      </c>
+      <c r="K25" s="3">
+        <f>J25/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>FINAL COST (with TP):</t>
+        </is>
+      </c>
+      <c r="B26" s="26">
+        <f>SUM(B19:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="16">
+        <f>B26/$B$9</f>
+        <v/>
+      </c>
+      <c r="D26" s="13">
+        <f>SUM(D19:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="14">
+        <f>D26/$B$9</f>
+        <v/>
+      </c>
+      <c r="F26" s="13">
+        <f>SUM(F19:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="14">
+        <f>F26/$B$9</f>
+        <v/>
+      </c>
+      <c r="H26" s="13">
+        <f>SUM(H19:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="14">
+        <f>H26/$B$9</f>
+        <v/>
+      </c>
+      <c r="J26" s="13">
+        <f>SUM(J19:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="14">
+        <f>J26/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Base for margin (Final Cost - TP)</t>
+        </is>
+      </c>
+      <c r="B27" s="24">
+        <f>B26-B21</f>
+        <v/>
+      </c>
+      <c r="C27" s="25">
+        <f>B27/$B$9</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>D26-D21</f>
+        <v/>
+      </c>
+      <c r="E27" s="3">
+        <f>D27/$B$9</f>
+        <v/>
+      </c>
+      <c r="F27" s="4">
+        <f>F26-F21</f>
+        <v/>
+      </c>
+      <c r="G27" s="3">
+        <f>F27/$B$9</f>
+        <v/>
+      </c>
+      <c r="H27" s="4">
+        <f>H26-H21</f>
+        <v/>
+      </c>
+      <c r="I27" s="3">
+        <f>H27/$B$9</f>
+        <v/>
+      </c>
+      <c r="J27" s="4">
+        <f>J26-J21</f>
+        <v/>
+      </c>
+      <c r="K27" s="3">
+        <f>J27/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Net price w/o TP (Base / (1 - TDM))</t>
+        </is>
+      </c>
+      <c r="B28" s="24">
+        <f>B27/(1-$B$10)</f>
+        <v/>
+      </c>
+      <c r="C28" s="25">
+        <f>B28/$B$9</f>
+        <v/>
+      </c>
+      <c r="D28" s="4">
+        <f>D27/(1-$B$10)</f>
+        <v/>
+      </c>
+      <c r="E28" s="3">
+        <f>D28/$B$9</f>
+        <v/>
+      </c>
+      <c r="F28" s="4">
+        <f>F27/(1-$B$10)</f>
+        <v/>
+      </c>
+      <c r="G28" s="3">
+        <f>F28/$B$9</f>
+        <v/>
+      </c>
+      <c r="H28" s="4">
+        <f>H27/(1-$B$10)</f>
+        <v/>
+      </c>
+      <c r="I28" s="3">
+        <f>H28/$B$9</f>
+        <v/>
+      </c>
+      <c r="J28" s="4">
+        <f>J27/(1-$B$10)</f>
+        <v/>
+      </c>
+      <c r="K28" s="3">
+        <f>J28/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>NET PRICE ('OUR PRICE'):</t>
+        </is>
+      </c>
+      <c r="B29" s="26">
+        <f>B28+B21</f>
+        <v/>
+      </c>
+      <c r="C29" s="16">
+        <f>B29/$B$9</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>D28+D21</f>
+        <v/>
+      </c>
+      <c r="E29" s="14">
+        <f>D29/$B$9</f>
+        <v/>
+      </c>
+      <c r="F29" s="13">
+        <f>F28+F21</f>
+        <v/>
+      </c>
+      <c r="G29" s="14">
+        <f>F29/$B$9</f>
+        <v/>
+      </c>
+      <c r="H29" s="13">
+        <f>H28+H21</f>
+        <v/>
+      </c>
+      <c r="I29" s="14">
+        <f>H29/$B$9</f>
+        <v/>
+      </c>
+      <c r="J29" s="13">
+        <f>J28+J21</f>
+        <v/>
+      </c>
+      <c r="K29" s="14">
+        <f>J29/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>+ PIS/COFINS (gross-up)</t>
+        </is>
+      </c>
+      <c r="B30" s="24">
+        <f>B29/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="C30" s="25">
+        <f>B30/$B$9</f>
+        <v/>
+      </c>
+      <c r="D30" s="4">
+        <f>D29/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="E30" s="3">
+        <f>D30/$B$9</f>
+        <v/>
+      </c>
+      <c r="F30" s="4">
+        <f>F29/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="G30" s="3">
+        <f>F30/$B$9</f>
+        <v/>
+      </c>
+      <c r="H30" s="4">
+        <f>H29/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="I30" s="3">
+        <f>H30/$B$9</f>
+        <v/>
+      </c>
+      <c r="J30" s="4">
+        <f>J29/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="K30" s="3">
+        <f>J30/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>+ ICMS (gross-up)</t>
+        </is>
+      </c>
+      <c r="B31" s="24">
+        <f>B30/(1-$B$12)</f>
+        <v/>
+      </c>
+      <c r="C31" s="25">
+        <f>B31/$B$9</f>
+        <v/>
+      </c>
+      <c r="D31" s="4">
+        <f>D30/(1-$B$12)</f>
+        <v/>
+      </c>
+      <c r="E31" s="3">
+        <f>D31/$B$9</f>
+        <v/>
+      </c>
+      <c r="F31" s="4">
+        <f>F30/(1-$B$12)</f>
+        <v/>
+      </c>
+      <c r="G31" s="3">
+        <f>F31/$B$9</f>
+        <v/>
+      </c>
+      <c r="H31" s="4">
+        <f>H30/(1-$B$12)</f>
+        <v/>
+      </c>
+      <c r="I31" s="3">
+        <f>H31/$B$9</f>
+        <v/>
+      </c>
+      <c r="J31" s="4">
+        <f>J30/(1-$B$12)</f>
+        <v/>
+      </c>
+      <c r="K31" s="3">
+        <f>J31/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>+ IPI (on top)</t>
+        </is>
+      </c>
+      <c r="B32" s="24">
+        <f>B31*$B$13</f>
+        <v/>
+      </c>
+      <c r="C32" s="25">
+        <f>B32/$B$9</f>
+        <v/>
+      </c>
+      <c r="D32" s="4">
+        <f>D31*$B$13</f>
+        <v/>
+      </c>
+      <c r="E32" s="3">
+        <f>D32/$B$9</f>
+        <v/>
+      </c>
+      <c r="F32" s="4">
+        <f>F31*$B$13</f>
+        <v/>
+      </c>
+      <c r="G32" s="3">
+        <f>F32/$B$9</f>
+        <v/>
+      </c>
+      <c r="H32" s="4">
+        <f>H31*$B$13</f>
+        <v/>
+      </c>
+      <c r="I32" s="3">
+        <f>H32/$B$9</f>
+        <v/>
+      </c>
+      <c r="J32" s="4">
+        <f>J31*$B$13</f>
+        <v/>
+      </c>
+      <c r="K32" s="3">
+        <f>J32/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>FINAL CLIENT PRICE:</t>
+        </is>
+      </c>
+      <c r="B33" s="26">
+        <f>B31+B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="16">
+        <f>B33/$B$9</f>
+        <v/>
+      </c>
+      <c r="D33" s="13">
+        <f>D31+D32</f>
+        <v/>
+      </c>
+      <c r="E33" s="14">
+        <f>D33/$B$9</f>
+        <v/>
+      </c>
+      <c r="F33" s="13">
+        <f>F31+F32</f>
+        <v/>
+      </c>
+      <c r="G33" s="14">
+        <f>F33/$B$9</f>
+        <v/>
+      </c>
+      <c r="H33" s="13">
+        <f>H31+H32</f>
+        <v/>
+      </c>
+      <c r="I33" s="14">
+        <f>H33/$B$9</f>
+        <v/>
+      </c>
+      <c r="J33" s="13">
+        <f>J31+J32</f>
+        <v/>
+      </c>
+      <c r="K33" s="14">
+        <f>J33/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>WHAT DRIVES THE FINAL CLIENT PRICE  (base case)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Removing ALL import duty (II) lowers the Final Client Price by</t>
+        </is>
+      </c>
+      <c r="B37" s="27">
+        <f>D33-F33</f>
+        <v/>
+      </c>
+      <c r="C37" s="3">
+        <f>B37/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Local output taxes (PIS/COFINS + ICMS + IPI) add on top of Net Price</t>
+        </is>
+      </c>
+      <c r="B38" s="27">
+        <f>D33-D29</f>
+        <v/>
+      </c>
+      <c r="C38" s="3">
+        <f>B38/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Local taxes are how many times bigger than the II effect?</t>
+        </is>
+      </c>
+      <c r="B39" s="28">
+        <f>B38/B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Final Client Price with NO II and 1 battery set, vs. US reference</t>
+        </is>
+      </c>
+      <c r="B40" s="21">
+        <f>J33/$B$9</f>
+        <v/>
+      </c>
+      <c r="C40" s="17">
+        <f>B40/$B$14-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>- II (import duty) sits inside the cost, so it is multiplied by the margin (1/(1-TDM)) and then by the local tax cascade - removing it is worth about 2.7x its face value in the final price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>- Even so, the local output taxes (PIS/COFINS, ICMS, IPI) stack on the whole price and outweigh the II effect - that is the point of this tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>- Battery sets: II, TP and freight of the batteries scale with the quantity; the row values come from the Final Cost List (84A222059P5, group without historical TP -&gt; 17.2%, no confirmed NCM -&gt; II 18%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>BASE VALUES (read from the P&amp;L tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1">
+      <c r="B47" s="29" t="inlineStr">
+        <is>
+          <t>Imported items, excluding batteries</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>Batteries - value per set (current BOM has 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Raw cost - imported items</t>
+        </is>
+      </c>
+      <c r="B48" s="4">
+        <f>'Executive Summary (P&amp;L)'!B10-2*C48</f>
+        <v/>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>79995.64</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Raw cost - PAC items</t>
+        </is>
+      </c>
+      <c r="B49" s="4">
+        <f>'Executive Summary (P&amp;L)'!B11</f>
+        <v/>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TP - Transfer Price</t>
+        </is>
+      </c>
+      <c r="B50" s="4">
+        <f>'Executive Summary (P&amp;L)'!B12-2*C50</f>
+        <v/>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>13759.25</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>International freight</t>
+        </is>
+      </c>
+      <c r="B51" s="4">
+        <f>'Executive Summary (P&amp;L)'!B13-2*C51</f>
+        <v/>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>1152.78</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>II - Import duty</t>
+        </is>
+      </c>
+      <c r="B52" s="4">
+        <f>'Executive Summary (P&amp;L)'!B14-2*C52</f>
+        <v/>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>17083.38</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Domestic freight</t>
+        </is>
+      </c>
+      <c r="B53" s="4">
+        <f>'Executive Summary (P&amp;L)'!B15</f>
+        <v/>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Supermetal - refurbishment / integration</t>
+        </is>
+      </c>
+      <c r="B54" s="4">
+        <f>'Executive Summary (P&amp;L)'!B16</f>
+        <v/>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A44:H44"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"0,1"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"1,2"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Make the finished-US-unit reference live now that its source file is in the repo
Matheus committed 'Planilha de Custos de Importacao - Pathfinder
completo- Set 26.xlsx' (sheet 'Pathfinder Pronto'), which
build_simulation_slide.py depends on - confirmed it now runs cleanly
here (previously failed with FileNotFoundError).

add_simulation_sheet.py's section 6 no longer hardcodes the 5
transcribed values; it reads H24/I22/I26/I27/I28/I35/I56 live from
that workbook, same as the slide does. Numbers match the slide within
rounding (total US$1,713,031 vs the slide's rounded US$1,713,000).
Re-verified zero formula/merge corruption in both summary workbooks.

README updated to point at the live source and restate the headline
finding: the landed finished-unit price is more expensive than all 4
build-via-Wabtec-Brasil scenarios.
</commit_message>
<xml_diff>
--- a/Pathfinder_Cost_Summary_EN.xlsx
+++ b/Pathfinder_Cost_Summary_EN.xlsx
@@ -10771,7 +10771,7 @@
         <v/>
       </c>
       <c r="C61" s="3" t="n">
-        <v>900000</v>
+        <v>899999.9999999999</v>
       </c>
     </row>
     <row r="62">
@@ -10785,7 +10785,7 @@
         <v/>
       </c>
       <c r="C62" s="3" t="n">
-        <v>80500</v>
+        <v>80490</v>
       </c>
     </row>
     <row r="63">
@@ -10799,7 +10799,7 @@
         <v/>
       </c>
       <c r="C63" s="3" t="n">
-        <v>16800</v>
+        <v>16842.85660194175</v>
       </c>
     </row>
     <row r="64">
@@ -10813,7 +10813,7 @@
         <v/>
       </c>
       <c r="C64" s="3" t="n">
-        <v>715700</v>
+        <v>715697.9140243899</v>
       </c>
     </row>
     <row r="65">
@@ -10885,7 +10885,7 @@
     <row r="73" ht="60" customHeight="1" s="31">
       <c r="A73" s="51" t="inlineStr">
         <is>
-          <t>- Source: 'Planilha de Custos de Importacao - Pathfinder completo- Set 26.xlsx' (sheet 'Pathfinder Pronto') - this workbook is NOT in the repo, so these 5 values are transcribed from the footnote of MRS_Pathfinder_Simulation_Local_Taxes_Bilingual.pptx, not computed live. Different scope than the 4 scenarios above: this is a finished, already-built unit (no Wabtec Brasil margin, no TP, no Supermetal refurbishment - it's a straight import of a complete product), so it is not an apples-to-apples 5th column of the scenario table. Get the source workbook to make this row live.</t>
+          <t>- Source: read LIVE from 'Planilha de Custos de Importacao - Pathfinder completo- Set 26.xlsx', sheet 'Pathfinder Pronto' (cells H24, I22, I26, I27, I28, I35, I56). Different scope than the 4 scenarios above: this is a finished, already-built unit (no Wabtec Brasil margin, no TP, no Supermetal refurbishment - it's a straight import of a complete product), so it is not an apples-to-apples 5th column of the scenario table.</t>
         </is>
       </c>
     </row>

</xml_diff>